<commit_message>
update excel file format
</commit_message>
<xml_diff>
--- a/templates/PhieuKetQuaChuKy.xlsx
+++ b/templates/PhieuKetQuaChuKy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/congdat/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/congdat/Developer/lab-admin-go/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5DB34D1-9410-774F-99FF-E4AAA8EC3502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C6FA33D-6469-E541-B6EC-28C404CFDA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5580" yWindow="2300" windowWidth="27640" windowHeight="16940" xr2:uid="{0D559CD5-B2C1-804F-9504-0EC5D04252A1}"/>
+    <workbookView xWindow="2600" yWindow="2300" windowWidth="27640" windowHeight="16940" xr2:uid="{0D559CD5-B2C1-804F-9504-0EC5D04252A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -348,20 +348,8 @@
   <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -372,22 +360,13 @@
     <xf numFmtId="14" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -430,6 +409,27 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -592,8 +592,8 @@
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>88900</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -623,8 +623,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="4203700" y="5842000"/>
-          <a:ext cx="3022600" cy="1371600"/>
+          <a:off x="4203700" y="3251200"/>
+          <a:ext cx="3632200" cy="1790700"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1497,328 +1497,328 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1">
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1">
       <c r="B2"/>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
     </row>
     <row r="3" spans="1:7" ht="6.75" customHeight="1">
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
     </row>
     <row r="4" spans="1:7" ht="18" customHeight="1">
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
     </row>
     <row r="5" spans="1:7" ht="18" customHeight="1">
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
     </row>
     <row r="6" spans="1:7" ht="10.5" customHeight="1">
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
     </row>
     <row r="7" spans="1:7" ht="24" customHeight="1">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
+      <c r="B7" s="38"/>
+      <c r="C7" s="38"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="38"/>
+      <c r="F7" s="38"/>
     </row>
     <row r="8" spans="1:7" ht="5.25" customHeight="1">
-      <c r="A8" s="8"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-    </row>
-    <row r="9" spans="1:7" s="9" customFormat="1" ht="18" customHeight="1">
-      <c r="B9" s="12" t="s">
+      <c r="A8" s="4"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+    </row>
+    <row r="9" spans="1:7" s="5" customFormat="1" ht="18" customHeight="1">
+      <c r="B9" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="9">
         <v>45778</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="F9" s="14"/>
-    </row>
-    <row r="10" spans="1:7" s="9" customFormat="1" ht="18" customHeight="1">
-      <c r="B10" s="12" t="s">
+      <c r="F9" s="39"/>
+    </row>
+    <row r="10" spans="1:7" s="5" customFormat="1" ht="18" customHeight="1">
+      <c r="B10" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E10" s="16">
+      <c r="E10" s="33">
         <v>1964</v>
       </c>
-      <c r="F10" s="16"/>
-    </row>
-    <row r="11" spans="1:7" s="9" customFormat="1" ht="18" customHeight="1">
-      <c r="B11" s="12" t="s">
+      <c r="F10" s="33"/>
+    </row>
+    <row r="11" spans="1:7" s="5" customFormat="1" ht="18" customHeight="1">
+      <c r="B11" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="16"/>
-    </row>
-    <row r="12" spans="1:7" s="20" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A12" s="18"/>
-      <c r="B12" s="12" t="s">
+      <c r="F11" s="33"/>
+    </row>
+    <row r="12" spans="1:7" s="13" customFormat="1" ht="18.75" customHeight="1">
+      <c r="A12" s="12"/>
+      <c r="B12" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
     </row>
     <row r="13" spans="1:7" ht="4.5" customHeight="1">
-      <c r="A13" s="21"/>
-      <c r="B13" s="21"/>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
+      <c r="A13" s="14"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
     </row>
     <row r="14" spans="1:7" ht="30" customHeight="1">
-      <c r="A14" s="22"/>
-      <c r="B14" s="23" t="s">
+      <c r="A14" s="15"/>
+      <c r="B14" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="23" t="s">
+      <c r="C14" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="23" t="s">
+      <c r="D14" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="E14" s="23" t="s">
+      <c r="E14" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="F14" s="23" t="s">
+      <c r="F14" s="16" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:7" s="9" customFormat="1" ht="17.5" customHeight="1">
-      <c r="A15" s="24"/>
-      <c r="B15" s="25"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="29" t="b">
+    <row r="15" spans="1:7" s="5" customFormat="1" ht="17.5" customHeight="1">
+      <c r="A15" s="17"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="22" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="18" customHeight="1">
-      <c r="B16" s="30"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="31"/>
-      <c r="F16" s="33"/>
-      <c r="G16" s="29"/>
+      <c r="B16" s="23"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="22"/>
     </row>
     <row r="17" spans="2:6" ht="18" customHeight="1">
-      <c r="B17" s="34"/>
-      <c r="C17" s="34"/>
-      <c r="D17" s="35"/>
-      <c r="E17" s="36"/>
-      <c r="F17" s="35"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="28"/>
     </row>
     <row r="18" spans="2:6" ht="18" customHeight="1">
-      <c r="B18" s="34"/>
-      <c r="C18" s="34"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="37"/>
+      <c r="B18" s="27"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="30"/>
     </row>
     <row r="19" spans="2:6" ht="18" customHeight="1">
-      <c r="B19" s="34"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="37"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="37"/>
+      <c r="B19" s="27"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="30"/>
     </row>
     <row r="20" spans="2:6" ht="18" customHeight="1">
-      <c r="B20" s="34"/>
-      <c r="C20" s="34"/>
-      <c r="D20" s="37"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="37"/>
+      <c r="B20" s="27"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="30"/>
     </row>
     <row r="21" spans="2:6" ht="18" customHeight="1">
-      <c r="B21" s="34"/>
-      <c r="C21" s="34"/>
-      <c r="D21" s="37"/>
-      <c r="E21" s="39"/>
-      <c r="F21" s="37"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="30"/>
     </row>
     <row r="22" spans="2:6" ht="18" customHeight="1">
-      <c r="B22" s="34"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="35"/>
+      <c r="B22" s="27"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="28"/>
     </row>
     <row r="23" spans="2:6" ht="18" customHeight="1">
-      <c r="B23" s="34"/>
-      <c r="C23" s="34"/>
-      <c r="E23" s="34"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="E23" s="27"/>
     </row>
     <row r="24" spans="2:6" ht="18" customHeight="1">
-      <c r="B24" s="34"/>
-      <c r="C24" s="34"/>
-      <c r="E24" s="34"/>
+      <c r="B24" s="27"/>
+      <c r="C24" s="27"/>
+      <c r="E24" s="27"/>
     </row>
     <row r="25" spans="2:6" ht="18" customHeight="1">
-      <c r="B25" s="34"/>
-      <c r="C25" s="34"/>
-      <c r="E25" s="34"/>
+      <c r="B25" s="27"/>
+      <c r="C25" s="27"/>
+      <c r="E25" s="27"/>
     </row>
     <row r="26" spans="2:6" ht="18" customHeight="1">
-      <c r="B26" s="34"/>
-      <c r="C26" s="34"/>
-      <c r="E26" s="34"/>
+      <c r="B26" s="27"/>
+      <c r="C26" s="27"/>
+      <c r="E26" s="27"/>
     </row>
     <row r="27" spans="2:6" ht="18" customHeight="1">
-      <c r="B27" s="34"/>
-      <c r="C27" s="34"/>
-      <c r="E27" s="34"/>
+      <c r="B27" s="27"/>
+      <c r="C27" s="27"/>
+      <c r="E27" s="27"/>
     </row>
     <row r="28" spans="2:6" ht="18" customHeight="1">
-      <c r="B28" s="34"/>
-      <c r="C28" s="34"/>
-      <c r="E28" s="34"/>
+      <c r="B28" s="27"/>
+      <c r="C28" s="27"/>
+      <c r="E28" s="27"/>
     </row>
     <row r="29" spans="2:6" ht="18" customHeight="1">
-      <c r="B29" s="34"/>
-      <c r="C29" s="34"/>
-      <c r="E29" s="34"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="27"/>
+      <c r="E29" s="27"/>
     </row>
     <row r="30" spans="2:6" ht="18" customHeight="1">
-      <c r="B30" s="34"/>
-      <c r="C30" s="34"/>
-      <c r="E30" s="34"/>
+      <c r="B30" s="27"/>
+      <c r="C30" s="27"/>
+      <c r="E30" s="27"/>
     </row>
     <row r="31" spans="2:6" ht="18" customHeight="1">
-      <c r="B31" s="34"/>
-      <c r="C31" s="34"/>
-      <c r="E31" s="34"/>
+      <c r="B31" s="27"/>
+      <c r="C31" s="27"/>
+      <c r="E31" s="27"/>
     </row>
     <row r="32" spans="2:6" ht="18" customHeight="1">
-      <c r="B32" s="34"/>
-      <c r="C32" s="34"/>
-      <c r="E32" s="34"/>
+      <c r="B32" s="27"/>
+      <c r="C32" s="27"/>
+      <c r="E32" s="27"/>
     </row>
     <row r="33" spans="2:5" ht="18" customHeight="1">
-      <c r="B33" s="34"/>
-      <c r="C33" s="34"/>
-      <c r="E33" s="34"/>
+      <c r="B33" s="27"/>
+      <c r="C33" s="27"/>
+      <c r="E33" s="27"/>
     </row>
     <row r="34" spans="2:5" ht="18" customHeight="1">
-      <c r="B34" s="34"/>
-      <c r="C34" s="34"/>
-      <c r="E34" s="34"/>
+      <c r="B34" s="27"/>
+      <c r="C34" s="27"/>
+      <c r="E34" s="27"/>
     </row>
     <row r="35" spans="2:5" ht="18" customHeight="1">
-      <c r="B35" s="34"/>
-      <c r="C35" s="34"/>
-      <c r="E35" s="34"/>
+      <c r="B35" s="27"/>
+      <c r="C35" s="27"/>
+      <c r="E35" s="27"/>
     </row>
     <row r="36" spans="2:5" ht="18" customHeight="1">
-      <c r="B36" s="34"/>
-      <c r="C36" s="34"/>
-      <c r="E36" s="34"/>
+      <c r="B36" s="27"/>
+      <c r="C36" s="27"/>
+      <c r="E36" s="27"/>
     </row>
     <row r="37" spans="2:5" ht="18" customHeight="1">
-      <c r="B37" s="34"/>
-      <c r="C37" s="34"/>
-      <c r="E37" s="34"/>
+      <c r="B37" s="27"/>
+      <c r="C37" s="27"/>
+      <c r="E37" s="27"/>
     </row>
     <row r="38" spans="2:5" ht="18" customHeight="1">
-      <c r="B38" s="34"/>
-      <c r="C38" s="34"/>
-      <c r="E38" s="34"/>
+      <c r="B38" s="27"/>
+      <c r="C38" s="27"/>
+      <c r="E38" s="27"/>
     </row>
     <row r="39" spans="2:5" ht="18" customHeight="1">
-      <c r="B39" s="34"/>
-      <c r="C39" s="34"/>
-      <c r="E39" s="34"/>
+      <c r="B39" s="27"/>
+      <c r="C39" s="27"/>
+      <c r="E39" s="27"/>
     </row>
     <row r="40" spans="2:5" ht="18" customHeight="1">
-      <c r="B40" s="34"/>
-      <c r="C40" s="34"/>
-      <c r="E40" s="34"/>
+      <c r="B40" s="27"/>
+      <c r="C40" s="27"/>
+      <c r="E40" s="27"/>
     </row>
     <row r="41" spans="2:5" ht="18" customHeight="1">
-      <c r="B41" s="34"/>
-      <c r="C41" s="34"/>
-      <c r="E41" s="34"/>
+      <c r="B41" s="27"/>
+      <c r="C41" s="27"/>
+      <c r="E41" s="27"/>
     </row>
     <row r="42" spans="2:5" ht="18" customHeight="1">
-      <c r="B42" s="34"/>
-      <c r="C42" s="34"/>
-      <c r="E42" s="34"/>
+      <c r="B42" s="27"/>
+      <c r="C42" s="27"/>
+      <c r="E42" s="27"/>
     </row>
     <row r="43" spans="2:5" ht="18" customHeight="1">
-      <c r="B43" s="34"/>
-      <c r="C43" s="34"/>
-      <c r="E43" s="34"/>
+      <c r="B43" s="27"/>
+      <c r="C43" s="27"/>
+      <c r="E43" s="27"/>
     </row>
     <row r="44" spans="2:5" ht="18" customHeight="1">
-      <c r="B44" s="34"/>
-      <c r="C44" s="34"/>
-      <c r="E44" s="34"/>
+      <c r="B44" s="27"/>
+      <c r="C44" s="27"/>
+      <c r="E44" s="27"/>
     </row>
     <row r="45" spans="2:5" ht="18" customHeight="1">
-      <c r="E45" s="34"/>
+      <c r="E45" s="27"/>
     </row>
     <row r="46" spans="2:5" ht="18" customHeight="1">
-      <c r="E46" s="34"/>
+      <c r="E46" s="27"/>
     </row>
     <row r="47" spans="2:5" ht="18" customHeight="1">
-      <c r="E47" s="34"/>
+      <c r="E47" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>

<commit_message>
feat: update excel file format (#25)
</commit_message>
<xml_diff>
--- a/templates/PhieuKetQuaChuKy.xlsx
+++ b/templates/PhieuKetQuaChuKy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/congdat/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/congdat/Developer/lab-admin-go/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5DB34D1-9410-774F-99FF-E4AAA8EC3502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C6FA33D-6469-E541-B6EC-28C404CFDA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5580" yWindow="2300" windowWidth="27640" windowHeight="16940" xr2:uid="{0D559CD5-B2C1-804F-9504-0EC5D04252A1}"/>
+    <workbookView xWindow="2600" yWindow="2300" windowWidth="27640" windowHeight="16940" xr2:uid="{0D559CD5-B2C1-804F-9504-0EC5D04252A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -348,20 +348,8 @@
   <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -372,22 +360,13 @@
     <xf numFmtId="14" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -430,6 +409,27 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -592,8 +592,8 @@
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>88900</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -623,8 +623,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="4203700" y="5842000"/>
-          <a:ext cx="3022600" cy="1371600"/>
+          <a:off x="4203700" y="3251200"/>
+          <a:ext cx="3632200" cy="1790700"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1497,328 +1497,328 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1">
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1">
       <c r="B2"/>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
     </row>
     <row r="3" spans="1:7" ht="6.75" customHeight="1">
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
     </row>
     <row r="4" spans="1:7" ht="18" customHeight="1">
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
     </row>
     <row r="5" spans="1:7" ht="18" customHeight="1">
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
     </row>
     <row r="6" spans="1:7" ht="10.5" customHeight="1">
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
     </row>
     <row r="7" spans="1:7" ht="24" customHeight="1">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
+      <c r="B7" s="38"/>
+      <c r="C7" s="38"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="38"/>
+      <c r="F7" s="38"/>
     </row>
     <row r="8" spans="1:7" ht="5.25" customHeight="1">
-      <c r="A8" s="8"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-    </row>
-    <row r="9" spans="1:7" s="9" customFormat="1" ht="18" customHeight="1">
-      <c r="B9" s="12" t="s">
+      <c r="A8" s="4"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+    </row>
+    <row r="9" spans="1:7" s="5" customFormat="1" ht="18" customHeight="1">
+      <c r="B9" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="9">
         <v>45778</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="F9" s="14"/>
-    </row>
-    <row r="10" spans="1:7" s="9" customFormat="1" ht="18" customHeight="1">
-      <c r="B10" s="12" t="s">
+      <c r="F9" s="39"/>
+    </row>
+    <row r="10" spans="1:7" s="5" customFormat="1" ht="18" customHeight="1">
+      <c r="B10" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E10" s="16">
+      <c r="E10" s="33">
         <v>1964</v>
       </c>
-      <c r="F10" s="16"/>
-    </row>
-    <row r="11" spans="1:7" s="9" customFormat="1" ht="18" customHeight="1">
-      <c r="B11" s="12" t="s">
+      <c r="F10" s="33"/>
+    </row>
+    <row r="11" spans="1:7" s="5" customFormat="1" ht="18" customHeight="1">
+      <c r="B11" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="16"/>
-    </row>
-    <row r="12" spans="1:7" s="20" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A12" s="18"/>
-      <c r="B12" s="12" t="s">
+      <c r="F11" s="33"/>
+    </row>
+    <row r="12" spans="1:7" s="13" customFormat="1" ht="18.75" customHeight="1">
+      <c r="A12" s="12"/>
+      <c r="B12" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
     </row>
     <row r="13" spans="1:7" ht="4.5" customHeight="1">
-      <c r="A13" s="21"/>
-      <c r="B13" s="21"/>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
+      <c r="A13" s="14"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
     </row>
     <row r="14" spans="1:7" ht="30" customHeight="1">
-      <c r="A14" s="22"/>
-      <c r="B14" s="23" t="s">
+      <c r="A14" s="15"/>
+      <c r="B14" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="23" t="s">
+      <c r="C14" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="23" t="s">
+      <c r="D14" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="E14" s="23" t="s">
+      <c r="E14" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="F14" s="23" t="s">
+      <c r="F14" s="16" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:7" s="9" customFormat="1" ht="17.5" customHeight="1">
-      <c r="A15" s="24"/>
-      <c r="B15" s="25"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="29" t="b">
+    <row r="15" spans="1:7" s="5" customFormat="1" ht="17.5" customHeight="1">
+      <c r="A15" s="17"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="22" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="18" customHeight="1">
-      <c r="B16" s="30"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="31"/>
-      <c r="F16" s="33"/>
-      <c r="G16" s="29"/>
+      <c r="B16" s="23"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="22"/>
     </row>
     <row r="17" spans="2:6" ht="18" customHeight="1">
-      <c r="B17" s="34"/>
-      <c r="C17" s="34"/>
-      <c r="D17" s="35"/>
-      <c r="E17" s="36"/>
-      <c r="F17" s="35"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="28"/>
     </row>
     <row r="18" spans="2:6" ht="18" customHeight="1">
-      <c r="B18" s="34"/>
-      <c r="C18" s="34"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="37"/>
+      <c r="B18" s="27"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="30"/>
     </row>
     <row r="19" spans="2:6" ht="18" customHeight="1">
-      <c r="B19" s="34"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="37"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="37"/>
+      <c r="B19" s="27"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="30"/>
     </row>
     <row r="20" spans="2:6" ht="18" customHeight="1">
-      <c r="B20" s="34"/>
-      <c r="C20" s="34"/>
-      <c r="D20" s="37"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="37"/>
+      <c r="B20" s="27"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="30"/>
     </row>
     <row r="21" spans="2:6" ht="18" customHeight="1">
-      <c r="B21" s="34"/>
-      <c r="C21" s="34"/>
-      <c r="D21" s="37"/>
-      <c r="E21" s="39"/>
-      <c r="F21" s="37"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="30"/>
     </row>
     <row r="22" spans="2:6" ht="18" customHeight="1">
-      <c r="B22" s="34"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="35"/>
+      <c r="B22" s="27"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="28"/>
     </row>
     <row r="23" spans="2:6" ht="18" customHeight="1">
-      <c r="B23" s="34"/>
-      <c r="C23" s="34"/>
-      <c r="E23" s="34"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="E23" s="27"/>
     </row>
     <row r="24" spans="2:6" ht="18" customHeight="1">
-      <c r="B24" s="34"/>
-      <c r="C24" s="34"/>
-      <c r="E24" s="34"/>
+      <c r="B24" s="27"/>
+      <c r="C24" s="27"/>
+      <c r="E24" s="27"/>
     </row>
     <row r="25" spans="2:6" ht="18" customHeight="1">
-      <c r="B25" s="34"/>
-      <c r="C25" s="34"/>
-      <c r="E25" s="34"/>
+      <c r="B25" s="27"/>
+      <c r="C25" s="27"/>
+      <c r="E25" s="27"/>
     </row>
     <row r="26" spans="2:6" ht="18" customHeight="1">
-      <c r="B26" s="34"/>
-      <c r="C26" s="34"/>
-      <c r="E26" s="34"/>
+      <c r="B26" s="27"/>
+      <c r="C26" s="27"/>
+      <c r="E26" s="27"/>
     </row>
     <row r="27" spans="2:6" ht="18" customHeight="1">
-      <c r="B27" s="34"/>
-      <c r="C27" s="34"/>
-      <c r="E27" s="34"/>
+      <c r="B27" s="27"/>
+      <c r="C27" s="27"/>
+      <c r="E27" s="27"/>
     </row>
     <row r="28" spans="2:6" ht="18" customHeight="1">
-      <c r="B28" s="34"/>
-      <c r="C28" s="34"/>
-      <c r="E28" s="34"/>
+      <c r="B28" s="27"/>
+      <c r="C28" s="27"/>
+      <c r="E28" s="27"/>
     </row>
     <row r="29" spans="2:6" ht="18" customHeight="1">
-      <c r="B29" s="34"/>
-      <c r="C29" s="34"/>
-      <c r="E29" s="34"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="27"/>
+      <c r="E29" s="27"/>
     </row>
     <row r="30" spans="2:6" ht="18" customHeight="1">
-      <c r="B30" s="34"/>
-      <c r="C30" s="34"/>
-      <c r="E30" s="34"/>
+      <c r="B30" s="27"/>
+      <c r="C30" s="27"/>
+      <c r="E30" s="27"/>
     </row>
     <row r="31" spans="2:6" ht="18" customHeight="1">
-      <c r="B31" s="34"/>
-      <c r="C31" s="34"/>
-      <c r="E31" s="34"/>
+      <c r="B31" s="27"/>
+      <c r="C31" s="27"/>
+      <c r="E31" s="27"/>
     </row>
     <row r="32" spans="2:6" ht="18" customHeight="1">
-      <c r="B32" s="34"/>
-      <c r="C32" s="34"/>
-      <c r="E32" s="34"/>
+      <c r="B32" s="27"/>
+      <c r="C32" s="27"/>
+      <c r="E32" s="27"/>
     </row>
     <row r="33" spans="2:5" ht="18" customHeight="1">
-      <c r="B33" s="34"/>
-      <c r="C33" s="34"/>
-      <c r="E33" s="34"/>
+      <c r="B33" s="27"/>
+      <c r="C33" s="27"/>
+      <c r="E33" s="27"/>
     </row>
     <row r="34" spans="2:5" ht="18" customHeight="1">
-      <c r="B34" s="34"/>
-      <c r="C34" s="34"/>
-      <c r="E34" s="34"/>
+      <c r="B34" s="27"/>
+      <c r="C34" s="27"/>
+      <c r="E34" s="27"/>
     </row>
     <row r="35" spans="2:5" ht="18" customHeight="1">
-      <c r="B35" s="34"/>
-      <c r="C35" s="34"/>
-      <c r="E35" s="34"/>
+      <c r="B35" s="27"/>
+      <c r="C35" s="27"/>
+      <c r="E35" s="27"/>
     </row>
     <row r="36" spans="2:5" ht="18" customHeight="1">
-      <c r="B36" s="34"/>
-      <c r="C36" s="34"/>
-      <c r="E36" s="34"/>
+      <c r="B36" s="27"/>
+      <c r="C36" s="27"/>
+      <c r="E36" s="27"/>
     </row>
     <row r="37" spans="2:5" ht="18" customHeight="1">
-      <c r="B37" s="34"/>
-      <c r="C37" s="34"/>
-      <c r="E37" s="34"/>
+      <c r="B37" s="27"/>
+      <c r="C37" s="27"/>
+      <c r="E37" s="27"/>
     </row>
     <row r="38" spans="2:5" ht="18" customHeight="1">
-      <c r="B38" s="34"/>
-      <c r="C38" s="34"/>
-      <c r="E38" s="34"/>
+      <c r="B38" s="27"/>
+      <c r="C38" s="27"/>
+      <c r="E38" s="27"/>
     </row>
     <row r="39" spans="2:5" ht="18" customHeight="1">
-      <c r="B39" s="34"/>
-      <c r="C39" s="34"/>
-      <c r="E39" s="34"/>
+      <c r="B39" s="27"/>
+      <c r="C39" s="27"/>
+      <c r="E39" s="27"/>
     </row>
     <row r="40" spans="2:5" ht="18" customHeight="1">
-      <c r="B40" s="34"/>
-      <c r="C40" s="34"/>
-      <c r="E40" s="34"/>
+      <c r="B40" s="27"/>
+      <c r="C40" s="27"/>
+      <c r="E40" s="27"/>
     </row>
     <row r="41" spans="2:5" ht="18" customHeight="1">
-      <c r="B41" s="34"/>
-      <c r="C41" s="34"/>
-      <c r="E41" s="34"/>
+      <c r="B41" s="27"/>
+      <c r="C41" s="27"/>
+      <c r="E41" s="27"/>
     </row>
     <row r="42" spans="2:5" ht="18" customHeight="1">
-      <c r="B42" s="34"/>
-      <c r="C42" s="34"/>
-      <c r="E42" s="34"/>
+      <c r="B42" s="27"/>
+      <c r="C42" s="27"/>
+      <c r="E42" s="27"/>
     </row>
     <row r="43" spans="2:5" ht="18" customHeight="1">
-      <c r="B43" s="34"/>
-      <c r="C43" s="34"/>
-      <c r="E43" s="34"/>
+      <c r="B43" s="27"/>
+      <c r="C43" s="27"/>
+      <c r="E43" s="27"/>
     </row>
     <row r="44" spans="2:5" ht="18" customHeight="1">
-      <c r="B44" s="34"/>
-      <c r="C44" s="34"/>
-      <c r="E44" s="34"/>
+      <c r="B44" s="27"/>
+      <c r="C44" s="27"/>
+      <c r="E44" s="27"/>
     </row>
     <row r="45" spans="2:5" ht="18" customHeight="1">
-      <c r="E45" s="34"/>
+      <c r="E45" s="27"/>
     </row>
     <row r="46" spans="2:5" ht="18" customHeight="1">
-      <c r="E46" s="34"/>
+      <c r="E46" s="27"/>
     </row>
     <row r="47" spans="2:5" ht="18" customHeight="1">
-      <c r="E47" s="34"/>
+      <c r="E47" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>

<commit_message>
refactor code and fix report format
</commit_message>
<xml_diff>
--- a/templates/PhieuKetQuaChuKy.xlsx
+++ b/templates/PhieuKetQuaChuKy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/congdat/Developer/lab-admin-go/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE63B84A-31FF-204A-BABD-0739B9EE5A36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0861068B-7017-2344-99B0-1A597C0F1E1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2600" yWindow="2300" windowWidth="27640" windowHeight="16940" xr2:uid="{0D559CD5-B2C1-804F-9504-0EC5D04252A1}"/>
   </bookViews>
@@ -165,7 +165,7 @@
     <t xml:space="preserve">                      PHÒNG XÉT NGHIỆM Y KHOA ANH QUÂN</t>
   </si>
   <si>
-    <t xml:space="preserve">                                       60 Đống Đa, Phường 2, TP. Cao Lãnh, Đồng Tháp.</t>
+    <t xml:space="preserve">                                             60 Đống Đa, Phường Cao Lãnh, Đồng Tháp.</t>
   </si>
 </sst>
 </file>
@@ -404,35 +404,35 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1502,27 +1502,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1">
-      <c r="C1" s="29" t="s">
+      <c r="C1" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1">
       <c r="B2"/>
-      <c r="C2" s="30" t="s">
+      <c r="C2" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
     </row>
     <row r="3" spans="1:7" ht="6.75" customHeight="1">
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
     </row>
     <row r="4" spans="1:7" ht="18" customHeight="1">
       <c r="C4" s="2" t="s">
@@ -1547,14 +1547,14 @@
       <c r="F6" s="3"/>
     </row>
     <row r="7" spans="1:7" ht="24" customHeight="1">
-      <c r="A7" s="32" t="s">
+      <c r="A7" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="32"/>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
+      <c r="B7" s="38"/>
+      <c r="C7" s="38"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="38"/>
+      <c r="F7" s="38"/>
     </row>
     <row r="8" spans="1:7" ht="5.25" customHeight="1">
       <c r="A8" s="4"/>
@@ -1565,59 +1565,59 @@
       <c r="F8" s="7"/>
     </row>
     <row r="9" spans="1:7" s="5" customFormat="1" ht="18" customHeight="1">
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="C9" s="34">
+      <c r="C9" s="30">
         <v>45778</v>
       </c>
-      <c r="D9" s="33" t="s">
+      <c r="D9" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="E9" s="35" t="s">
+      <c r="E9" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="F9" s="35"/>
+      <c r="F9" s="39"/>
     </row>
     <row r="10" spans="1:7" s="5" customFormat="1" ht="18" customHeight="1">
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="36" t="s">
+      <c r="C10" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="33" t="s">
+      <c r="D10" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="E10" s="37">
+      <c r="E10" s="33">
         <v>1964</v>
       </c>
-      <c r="F10" s="37"/>
+      <c r="F10" s="33"/>
     </row>
     <row r="11" spans="1:7" s="5" customFormat="1" ht="18" customHeight="1">
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="38" t="s">
+      <c r="C11" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="33" t="s">
+      <c r="D11" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="37" t="s">
+      <c r="E11" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="F11" s="37"/>
+      <c r="F11" s="33"/>
     </row>
     <row r="12" spans="1:7" s="9" customFormat="1" ht="18.75" customHeight="1">
       <c r="A12" s="8"/>
-      <c r="B12" s="33" t="s">
+      <c r="B12" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
     </row>
     <row r="13" spans="1:7" ht="4.5" customHeight="1">
       <c r="A13" s="10"/>

</xml_diff>

<commit_message>
fix: bug test order in tracking page and update record format (#48)
* fix bug test order in tracking page

* refactor code and fix report format

* refactor code to reduce duplication in style init
</commit_message>
<xml_diff>
--- a/templates/PhieuKetQuaChuKy.xlsx
+++ b/templates/PhieuKetQuaChuKy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/congdat/Developer/lab-admin-go/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE63B84A-31FF-204A-BABD-0739B9EE5A36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0861068B-7017-2344-99B0-1A597C0F1E1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2600" yWindow="2300" windowWidth="27640" windowHeight="16940" xr2:uid="{0D559CD5-B2C1-804F-9504-0EC5D04252A1}"/>
   </bookViews>
@@ -165,7 +165,7 @@
     <t xml:space="preserve">                      PHÒNG XÉT NGHIỆM Y KHOA ANH QUÂN</t>
   </si>
   <si>
-    <t xml:space="preserve">                                       60 Đống Đa, Phường 2, TP. Cao Lãnh, Đồng Tháp.</t>
+    <t xml:space="preserve">                                             60 Đống Đa, Phường Cao Lãnh, Đồng Tháp.</t>
   </si>
 </sst>
 </file>
@@ -404,35 +404,35 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1502,27 +1502,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1">
-      <c r="C1" s="29" t="s">
+      <c r="C1" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1">
       <c r="B2"/>
-      <c r="C2" s="30" t="s">
+      <c r="C2" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
     </row>
     <row r="3" spans="1:7" ht="6.75" customHeight="1">
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
     </row>
     <row r="4" spans="1:7" ht="18" customHeight="1">
       <c r="C4" s="2" t="s">
@@ -1547,14 +1547,14 @@
       <c r="F6" s="3"/>
     </row>
     <row r="7" spans="1:7" ht="24" customHeight="1">
-      <c r="A7" s="32" t="s">
+      <c r="A7" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="32"/>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
+      <c r="B7" s="38"/>
+      <c r="C7" s="38"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="38"/>
+      <c r="F7" s="38"/>
     </row>
     <row r="8" spans="1:7" ht="5.25" customHeight="1">
       <c r="A8" s="4"/>
@@ -1565,59 +1565,59 @@
       <c r="F8" s="7"/>
     </row>
     <row r="9" spans="1:7" s="5" customFormat="1" ht="18" customHeight="1">
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="C9" s="34">
+      <c r="C9" s="30">
         <v>45778</v>
       </c>
-      <c r="D9" s="33" t="s">
+      <c r="D9" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="E9" s="35" t="s">
+      <c r="E9" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="F9" s="35"/>
+      <c r="F9" s="39"/>
     </row>
     <row r="10" spans="1:7" s="5" customFormat="1" ht="18" customHeight="1">
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="36" t="s">
+      <c r="C10" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="33" t="s">
+      <c r="D10" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="E10" s="37">
+      <c r="E10" s="33">
         <v>1964</v>
       </c>
-      <c r="F10" s="37"/>
+      <c r="F10" s="33"/>
     </row>
     <row r="11" spans="1:7" s="5" customFormat="1" ht="18" customHeight="1">
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="38" t="s">
+      <c r="C11" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="33" t="s">
+      <c r="D11" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="37" t="s">
+      <c r="E11" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="F11" s="37"/>
+      <c r="F11" s="33"/>
     </row>
     <row r="12" spans="1:7" s="9" customFormat="1" ht="18.75" customHeight="1">
       <c r="A12" s="8"/>
-      <c r="B12" s="33" t="s">
+      <c r="B12" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
     </row>
     <row r="13" spans="1:7" ht="4.5" customHeight="1">
       <c r="A13" s="10"/>

</xml_diff>